<commit_message>
Use a single green color scheme in the literature matrix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QgqFT5Fkzz2mf4ivKRGXX
</commit_message>
<xml_diff>
--- a/downloads/Literature_Matrix_Burnout_Sleep_Recovery_Women.xlsx
+++ b/downloads/Literature_Matrix_Burnout_Sleep_Recovery_Women.xlsx
@@ -3250,7 +3250,7 @@
     <font>
       <b val="true"/>
       <sz val="14"/>
-      <color rgb="FF1F3A5F"/>
+      <color rgb="FF1E5631"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -3287,7 +3287,7 @@
     <font>
       <u val="single"/>
       <sz val="10"/>
-      <color rgb="FF0563C1"/>
+      <color rgb="FF1E5631"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -3302,13 +3302,13 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF7A1F1F"/>
+      <color rgb="FF1E5631"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3317,43 +3317,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F3A5F"/>
+        <fgColor rgb="FF1E5631"/>
         <bgColor rgb="FF274E13"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2E5C8A"/>
-        <bgColor rgb="FF5B4B8A"/>
+        <fgColor rgb="FF2E7D32"/>
+        <bgColor rgb="FF008000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF3B7A57"/>
-        <bgColor rgb="FF2E5C8A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF7A4B2E"/>
-        <bgColor rgb="FF555555"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF5B4B8A"/>
-        <bgColor rgb="FF555555"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF555555"/>
-        <bgColor rgb="FF5B4B8A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF3F6FA"/>
+        <fgColor rgb="FFF1F8F1"/>
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
@@ -3407,7 +3383,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3441,46 +3417,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3492,19 +3428,19 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3512,7 +3448,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3565,11 +3501,11 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF1F3A5F"/>
+          <fgColor rgb="FF2E7D32"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -3577,7 +3513,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF3F6FA"/>
+          <fgColor rgb="FFF1F8F1"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -3600,39 +3536,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF2E5C8A"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF3B7A57"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF7A4B2E"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF5B4B8A"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9EAD3"/>
+          <fgColor rgb="FFC8E6C9"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -3648,15 +3552,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF555555"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF0563C1"/>
+          <fgColor rgb="FF1E5631"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -3671,7 +3567,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFC8E6C9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3695,12 +3591,12 @@
       <rgbColor rgb="FFBFBFBF"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF7A4B2E"/>
-      <rgbColor rgb="FFF3F6FA"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFF1F8F1"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0563C1"/>
+      <rgbColor rgb="FF0066CC"/>
       <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -3712,7 +3608,7 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFD9EAD3"/>
+      <rgbColor rgb="FFC8E6C9"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
@@ -3724,16 +3620,16 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF5B4B8A"/>
+      <rgbColor rgb="FF555555"/>
       <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF1F3A5F"/>
-      <rgbColor rgb="FF3B7A57"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF2E7D32"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF274E13"/>
-      <rgbColor rgb="FF7A1F1F"/>
+      <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF2E5C8A"/>
-      <rgbColor rgb="FF555555"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF1E5631"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -4148,134 +4044,134 @@
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="9" t="s">
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="10" t="s">
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
-      <c r="S3" s="10"/>
-      <c r="T3" s="11" t="s">
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="U3" s="11"/>
-      <c r="V3" s="11"/>
-      <c r="W3" s="11"/>
-      <c r="X3" s="11"/>
-      <c r="Y3" s="11"/>
-      <c r="Z3" s="12" t="s">
+      <c r="U3" s="7"/>
+      <c r="V3" s="7"/>
+      <c r="W3" s="7"/>
+      <c r="X3" s="7"/>
+      <c r="Y3" s="7"/>
+      <c r="Z3" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="AA3" s="12"/>
-      <c r="AB3" s="12"/>
+      <c r="AA3" s="7"/>
+      <c r="AB3" s="7"/>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="14" t="s">
+      <c r="H4" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I4" s="14" t="s">
+      <c r="I4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="14" t="s">
+      <c r="J4" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="K4" s="14" t="s">
+      <c r="K4" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="L4" s="15" t="s">
+      <c r="L4" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="M4" s="15" t="s">
+      <c r="M4" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="N4" s="15" t="s">
+      <c r="N4" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="O4" s="15" t="s">
+      <c r="O4" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="P4" s="16" t="s">
+      <c r="P4" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="Q4" s="16" t="s">
+      <c r="Q4" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="R4" s="16" t="s">
+      <c r="R4" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="S4" s="16" t="s">
+      <c r="S4" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="T4" s="17" t="s">
+      <c r="T4" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="U4" s="17" t="s">
+      <c r="U4" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="V4" s="17" t="s">
+      <c r="V4" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="W4" s="17" t="s">
+      <c r="W4" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="X4" s="17" t="s">
+      <c r="X4" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="Y4" s="17" t="s">
+      <c r="Y4" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="Z4" s="18" t="s">
+      <c r="Z4" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="AA4" s="18" t="s">
+      <c r="AA4" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="AB4" s="18" t="s">
+      <c r="AB4" s="8" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="69" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="n">
+      <c r="A5" s="9" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="9" t="n">
         <v>2024</v>
       </c>
       <c r="D5" s="6" t="s">
@@ -4293,7 +4189,7 @@
       <c r="H5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I5" s="19" t="s">
+      <c r="I5" s="9" t="s">
         <v>75</v>
       </c>
       <c r="J5" s="6" t="s">
@@ -4326,16 +4222,16 @@
       <c r="S5" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="T5" s="19"/>
-      <c r="U5" s="19"/>
-      <c r="V5" s="19"/>
-      <c r="W5" s="19"/>
-      <c r="X5" s="19"/>
-      <c r="Y5" s="19"/>
+      <c r="T5" s="9"/>
+      <c r="U5" s="9"/>
+      <c r="V5" s="9"/>
+      <c r="W5" s="9"/>
+      <c r="X5" s="9"/>
+      <c r="Y5" s="9"/>
       <c r="Z5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="AA5" s="20" t="s">
+      <c r="AA5" s="10" t="s">
         <v>83</v>
       </c>
       <c r="AB5" s="6" t="s">
@@ -4343,91 +4239,91 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="n">
+      <c r="A6" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="11" t="n">
         <v>2023</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="F6" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="G6" s="22" t="s">
+      <c r="G6" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="H6" s="22" t="s">
+      <c r="H6" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="I6" s="21" t="s">
+      <c r="I6" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="22" t="s">
+      <c r="J6" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="K6" s="22" t="s">
+      <c r="K6" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="L6" s="22" t="s">
+      <c r="L6" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="M6" s="22" t="s">
+      <c r="M6" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="N6" s="22" t="s">
+      <c r="N6" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="O6" s="22" t="s">
+      <c r="O6" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="P6" s="22" t="s">
+      <c r="P6" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="Q6" s="22" t="s">
+      <c r="Q6" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="R6" s="22" t="s">
+      <c r="R6" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="S6" s="22" t="s">
+      <c r="S6" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="T6" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="U6" s="21"/>
-      <c r="V6" s="21"/>
-      <c r="W6" s="21"/>
-      <c r="X6" s="21"/>
-      <c r="Y6" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z6" s="23" t="n">
+      <c r="T6" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="U6" s="11"/>
+      <c r="V6" s="11"/>
+      <c r="W6" s="11"/>
+      <c r="X6" s="11"/>
+      <c r="Y6" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z6" s="13" t="n">
         <v>37651959</v>
       </c>
-      <c r="AA6" s="24" t="s">
+      <c r="AA6" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="AB6" s="22" t="s">
+      <c r="AB6" s="12" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="n">
+      <c r="A7" s="9" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="9" t="n">
         <v>2024</v>
       </c>
       <c r="D7" s="6" t="s">
@@ -4445,7 +4341,7 @@
       <c r="H7" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="I7" s="19" t="s">
+      <c r="I7" s="9" t="s">
         <v>16</v>
       </c>
       <c r="J7" s="6" t="s">
@@ -4478,20 +4374,20 @@
       <c r="S7" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="T7" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="U7" s="19"/>
-      <c r="V7" s="19"/>
-      <c r="W7" s="19"/>
-      <c r="X7" s="19"/>
-      <c r="Y7" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z7" s="25" t="n">
+      <c r="T7" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="U7" s="9"/>
+      <c r="V7" s="9"/>
+      <c r="W7" s="9"/>
+      <c r="X7" s="9"/>
+      <c r="Y7" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z7" s="15" t="n">
         <v>39120506</v>
       </c>
-      <c r="AA7" s="20" t="s">
+      <c r="AA7" s="10" t="s">
         <v>109</v>
       </c>
       <c r="AB7" s="6" t="s">
@@ -4499,91 +4395,91 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="n">
+      <c r="A8" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="11" t="n">
         <v>2021</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="D8" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="F8" s="22" t="s">
+      <c r="F8" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="G8" s="22" t="s">
+      <c r="G8" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="H8" s="22" t="s">
+      <c r="H8" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="I8" s="21" t="s">
+      <c r="I8" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="22" t="s">
+      <c r="J8" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="K8" s="22" t="s">
+      <c r="K8" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="L8" s="22" t="s">
+      <c r="L8" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="M8" s="22" t="s">
+      <c r="M8" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="N8" s="22" t="s">
+      <c r="N8" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="O8" s="22" t="s">
+      <c r="O8" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="P8" s="22" t="s">
+      <c r="P8" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="Q8" s="22" t="s">
+      <c r="Q8" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="R8" s="22" t="s">
+      <c r="R8" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="S8" s="22" t="s">
+      <c r="S8" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="T8" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="U8" s="21"/>
-      <c r="V8" s="21"/>
-      <c r="W8" s="21"/>
-      <c r="X8" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y8" s="21"/>
-      <c r="Z8" s="23" t="n">
+      <c r="T8" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="U8" s="11"/>
+      <c r="V8" s="11"/>
+      <c r="W8" s="11"/>
+      <c r="X8" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y8" s="11"/>
+      <c r="Z8" s="13" t="n">
         <v>34081678</v>
       </c>
-      <c r="AA8" s="24" t="s">
+      <c r="AA8" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="AB8" s="22" t="s">
+      <c r="AB8" s="12" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="n">
+      <c r="A9" s="9" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="C9" s="19" t="n">
+      <c r="C9" s="9" t="n">
         <v>2022</v>
       </c>
       <c r="D9" s="6" t="s">
@@ -4601,7 +4497,7 @@
       <c r="H9" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="I9" s="19" t="s">
+      <c r="I9" s="9" t="s">
         <v>16</v>
       </c>
       <c r="J9" s="6" t="s">
@@ -4634,22 +4530,22 @@
       <c r="S9" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="T9" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="U9" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="V9" s="19"/>
-      <c r="W9" s="19"/>
-      <c r="X9" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y9" s="19"/>
-      <c r="Z9" s="25" t="n">
+      <c r="T9" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="U9" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V9" s="9"/>
+      <c r="W9" s="9"/>
+      <c r="X9" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y9" s="9"/>
+      <c r="Z9" s="15" t="n">
         <v>35628091</v>
       </c>
-      <c r="AA9" s="20" t="s">
+      <c r="AA9" s="10" t="s">
         <v>136</v>
       </c>
       <c r="AB9" s="6" t="s">
@@ -4657,93 +4553,93 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="n">
+      <c r="A10" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="11" t="n">
         <v>2025</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="F10" s="22" t="s">
+      <c r="F10" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="G10" s="22" t="s">
+      <c r="G10" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="H10" s="22" t="s">
+      <c r="H10" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="I10" s="26" t="n">
+      <c r="I10" s="16" t="n">
         <v>0.664</v>
       </c>
-      <c r="J10" s="22" t="s">
+      <c r="J10" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="K10" s="22" t="s">
+      <c r="K10" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="L10" s="22" t="s">
+      <c r="L10" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="M10" s="22" t="s">
+      <c r="M10" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="N10" s="22" t="s">
+      <c r="N10" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="O10" s="22" t="s">
+      <c r="O10" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="P10" s="22" t="s">
+      <c r="P10" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="Q10" s="22" t="s">
+      <c r="Q10" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="R10" s="22" t="s">
+      <c r="R10" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="S10" s="22" t="s">
+      <c r="S10" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="T10" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="U10" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="V10" s="21"/>
-      <c r="W10" s="21"/>
-      <c r="X10" s="21"/>
-      <c r="Y10" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z10" s="23" t="n">
+      <c r="T10" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="U10" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="V10" s="11"/>
+      <c r="W10" s="11"/>
+      <c r="X10" s="11"/>
+      <c r="Y10" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z10" s="13" t="n">
         <v>40624657</v>
       </c>
-      <c r="AA10" s="24" t="s">
+      <c r="AA10" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="AB10" s="22" t="s">
+      <c r="AB10" s="12" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="n">
+      <c r="A11" s="9" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="C11" s="19" t="n">
+      <c r="C11" s="9" t="n">
         <v>2023</v>
       </c>
       <c r="D11" s="6" t="s">
@@ -4761,7 +4657,7 @@
       <c r="H11" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="I11" s="19" t="s">
+      <c r="I11" s="9" t="s">
         <v>14</v>
       </c>
       <c r="J11" s="6" t="s">
@@ -4794,22 +4690,22 @@
       <c r="S11" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="T11" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="U11" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="V11" s="19"/>
-      <c r="W11" s="19"/>
-      <c r="X11" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y11" s="19"/>
-      <c r="Z11" s="25" t="n">
+      <c r="T11" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="U11" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V11" s="9"/>
+      <c r="W11" s="9"/>
+      <c r="X11" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y11" s="9"/>
+      <c r="Z11" s="15" t="n">
         <v>36634111</v>
       </c>
-      <c r="AA11" s="20" t="s">
+      <c r="AA11" s="10" t="s">
         <v>166</v>
       </c>
       <c r="AB11" s="6" t="s">
@@ -4817,91 +4713,91 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="n">
+      <c r="A12" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="C12" s="21" t="n">
+      <c r="C12" s="11" t="n">
         <v>2025</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="E12" s="22" t="s">
+      <c r="E12" s="12" t="s">
         <v>170</v>
       </c>
-      <c r="F12" s="22" t="s">
+      <c r="F12" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="G12" s="22" t="s">
+      <c r="G12" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="H12" s="22" t="s">
+      <c r="H12" s="12" t="s">
         <v>172</v>
       </c>
-      <c r="I12" s="21" t="s">
+      <c r="I12" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="J12" s="22" t="s">
+      <c r="J12" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="K12" s="22" t="s">
+      <c r="K12" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="L12" s="22" t="s">
+      <c r="L12" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="M12" s="22" t="s">
+      <c r="M12" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="N12" s="22" t="s">
+      <c r="N12" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="O12" s="22" t="s">
+      <c r="O12" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="P12" s="22" t="s">
+      <c r="P12" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="Q12" s="22" t="s">
+      <c r="Q12" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="R12" s="22" t="s">
+      <c r="R12" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="S12" s="22" t="s">
+      <c r="S12" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="T12" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="U12" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="V12" s="21"/>
-      <c r="W12" s="21"/>
-      <c r="X12" s="21"/>
-      <c r="Y12" s="21"/>
-      <c r="Z12" s="23" t="n">
+      <c r="T12" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="U12" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="V12" s="11"/>
+      <c r="W12" s="11"/>
+      <c r="X12" s="11"/>
+      <c r="Y12" s="11"/>
+      <c r="Z12" s="13" t="n">
         <v>40659822</v>
       </c>
-      <c r="AA12" s="24" t="s">
+      <c r="AA12" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="AB12" s="22" t="s">
+      <c r="AB12" s="12" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="n">
+      <c r="A13" s="9" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="C13" s="19" t="n">
+      <c r="C13" s="9" t="n">
         <v>2025</v>
       </c>
       <c r="D13" s="6" t="s">
@@ -4919,7 +4815,7 @@
       <c r="H13" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="I13" s="19" t="s">
+      <c r="I13" s="9" t="s">
         <v>14</v>
       </c>
       <c r="J13" s="6" t="s">
@@ -4952,20 +4848,20 @@
       <c r="S13" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="T13" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="U13" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="V13" s="19"/>
-      <c r="W13" s="19"/>
-      <c r="X13" s="19"/>
-      <c r="Y13" s="19"/>
-      <c r="Z13" s="25" t="n">
+      <c r="T13" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="U13" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V13" s="9"/>
+      <c r="W13" s="9"/>
+      <c r="X13" s="9"/>
+      <c r="Y13" s="9"/>
+      <c r="Z13" s="15" t="n">
         <v>40328567</v>
       </c>
-      <c r="AA13" s="20" t="s">
+      <c r="AA13" s="10" t="s">
         <v>196</v>
       </c>
       <c r="AB13" s="6" t="s">
@@ -4973,91 +4869,91 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="n">
+      <c r="A14" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="12" t="s">
         <v>198</v>
       </c>
-      <c r="C14" s="21" t="n">
+      <c r="C14" s="11" t="n">
         <v>2021</v>
       </c>
-      <c r="D14" s="22" t="s">
+      <c r="D14" s="12" t="s">
         <v>199</v>
       </c>
-      <c r="E14" s="22" t="s">
+      <c r="E14" s="12" t="s">
         <v>200</v>
       </c>
-      <c r="F14" s="22" t="s">
+      <c r="F14" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="G14" s="22" t="s">
+      <c r="G14" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="H14" s="22" t="s">
+      <c r="H14" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="I14" s="21" t="s">
+      <c r="I14" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="J14" s="22" t="s">
+      <c r="J14" s="12" t="s">
         <v>204</v>
       </c>
-      <c r="K14" s="22" t="s">
+      <c r="K14" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="L14" s="22" t="s">
+      <c r="L14" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="M14" s="22" t="s">
+      <c r="M14" s="12" t="s">
         <v>206</v>
       </c>
-      <c r="N14" s="22" t="s">
+      <c r="N14" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="O14" s="22" t="s">
+      <c r="O14" s="12" t="s">
         <v>207</v>
       </c>
-      <c r="P14" s="22" t="s">
+      <c r="P14" s="12" t="s">
         <v>208</v>
       </c>
-      <c r="Q14" s="22" t="s">
+      <c r="Q14" s="12" t="s">
         <v>209</v>
       </c>
-      <c r="R14" s="22" t="s">
+      <c r="R14" s="12" t="s">
         <v>210</v>
       </c>
-      <c r="S14" s="22" t="s">
+      <c r="S14" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="T14" s="21"/>
-      <c r="U14" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="V14" s="21"/>
-      <c r="W14" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="X14" s="21"/>
-      <c r="Y14" s="21"/>
-      <c r="Z14" s="23" t="n">
+      <c r="T14" s="11"/>
+      <c r="U14" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="V14" s="11"/>
+      <c r="W14" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="X14" s="11"/>
+      <c r="Y14" s="11"/>
+      <c r="Z14" s="13" t="n">
         <v>33603132</v>
       </c>
-      <c r="AA14" s="24" t="s">
+      <c r="AA14" s="14" t="s">
         <v>211</v>
       </c>
-      <c r="AB14" s="22" t="s">
+      <c r="AB14" s="12" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="n">
+      <c r="A15" s="9" t="n">
         <v>11</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="C15" s="19" t="n">
+      <c r="C15" s="9" t="n">
         <v>2026</v>
       </c>
       <c r="D15" s="6" t="s">
@@ -5075,7 +4971,7 @@
       <c r="H15" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="I15" s="19" t="s">
+      <c r="I15" s="9" t="s">
         <v>14</v>
       </c>
       <c r="J15" s="6" t="s">
@@ -5108,20 +5004,20 @@
       <c r="S15" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="T15" s="19"/>
-      <c r="U15" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="V15" s="19"/>
-      <c r="W15" s="19"/>
-      <c r="X15" s="19"/>
-      <c r="Y15" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z15" s="25" t="n">
+      <c r="T15" s="9"/>
+      <c r="U15" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V15" s="9"/>
+      <c r="W15" s="9"/>
+      <c r="X15" s="9"/>
+      <c r="Y15" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z15" s="15" t="n">
         <v>42138024</v>
       </c>
-      <c r="AA15" s="20" t="s">
+      <c r="AA15" s="10" t="s">
         <v>224</v>
       </c>
       <c r="AB15" s="6" t="s">
@@ -5129,95 +5025,95 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="22" t="s">
+      <c r="A16" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="11" t="n">
         <v>2026</v>
       </c>
-      <c r="D16" s="22" t="s">
+      <c r="D16" s="12" t="s">
         <v>227</v>
       </c>
-      <c r="E16" s="22" t="s">
+      <c r="E16" s="12" t="s">
         <v>228</v>
       </c>
-      <c r="F16" s="22" t="s">
+      <c r="F16" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="G16" s="22" t="s">
+      <c r="G16" s="12" t="s">
         <v>229</v>
       </c>
-      <c r="H16" s="22" t="s">
+      <c r="H16" s="12" t="s">
         <v>230</v>
       </c>
-      <c r="I16" s="21" t="s">
+      <c r="I16" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="J16" s="22" t="s">
+      <c r="J16" s="12" t="s">
         <v>231</v>
       </c>
-      <c r="K16" s="22" t="s">
+      <c r="K16" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="L16" s="22" t="s">
+      <c r="L16" s="12" t="s">
         <v>232</v>
       </c>
-      <c r="M16" s="22" t="s">
+      <c r="M16" s="12" t="s">
         <v>233</v>
       </c>
-      <c r="N16" s="22" t="s">
+      <c r="N16" s="12" t="s">
         <v>234</v>
       </c>
-      <c r="O16" s="22" t="s">
+      <c r="O16" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="P16" s="22" t="s">
+      <c r="P16" s="12" t="s">
         <v>236</v>
       </c>
-      <c r="Q16" s="22" t="s">
+      <c r="Q16" s="12" t="s">
         <v>237</v>
       </c>
-      <c r="R16" s="22" t="s">
+      <c r="R16" s="12" t="s">
         <v>238</v>
       </c>
-      <c r="S16" s="22" t="s">
+      <c r="S16" s="12" t="s">
         <v>239</v>
       </c>
-      <c r="T16" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="U16" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="V16" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="W16" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="X16" s="21"/>
-      <c r="Y16" s="21"/>
-      <c r="Z16" s="23" t="n">
+      <c r="T16" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="U16" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="V16" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="W16" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="X16" s="11"/>
+      <c r="Y16" s="11"/>
+      <c r="Z16" s="13" t="n">
         <v>41591133</v>
       </c>
-      <c r="AA16" s="24" t="s">
+      <c r="AA16" s="14" t="s">
         <v>240</v>
       </c>
-      <c r="AB16" s="22" t="s">
+      <c r="AB16" s="12" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="n">
+      <c r="A17" s="9" t="n">
         <v>13</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="C17" s="19" t="n">
+      <c r="C17" s="9" t="n">
         <v>2025</v>
       </c>
       <c r="D17" s="6" t="s">
@@ -5235,7 +5131,7 @@
       <c r="H17" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="I17" s="19" t="s">
+      <c r="I17" s="9" t="s">
         <v>16</v>
       </c>
       <c r="J17" s="6" t="s">
@@ -5268,18 +5164,18 @@
       <c r="S17" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="T17" s="19"/>
-      <c r="U17" s="19"/>
-      <c r="V17" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="W17" s="19"/>
-      <c r="X17" s="19"/>
-      <c r="Y17" s="19"/>
-      <c r="Z17" s="25" t="n">
+      <c r="T17" s="9"/>
+      <c r="U17" s="9"/>
+      <c r="V17" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W17" s="9"/>
+      <c r="X17" s="9"/>
+      <c r="Y17" s="9"/>
+      <c r="Z17" s="15" t="n">
         <v>41157926</v>
       </c>
-      <c r="AA17" s="20" t="s">
+      <c r="AA17" s="10" t="s">
         <v>255</v>
       </c>
       <c r="AB17" s="6" t="s">
@@ -5287,93 +5183,93 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="n">
+      <c r="A18" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="12" t="s">
         <v>257</v>
       </c>
-      <c r="C18" s="21" t="n">
+      <c r="C18" s="11" t="n">
         <v>2026</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="12" t="s">
         <v>258</v>
       </c>
-      <c r="E18" s="22" t="s">
+      <c r="E18" s="12" t="s">
         <v>259</v>
       </c>
-      <c r="F18" s="22" t="s">
+      <c r="F18" s="12" t="s">
         <v>260</v>
       </c>
-      <c r="G18" s="22" t="s">
+      <c r="G18" s="12" t="s">
         <v>261</v>
       </c>
-      <c r="H18" s="22" t="s">
+      <c r="H18" s="12" t="s">
         <v>262</v>
       </c>
-      <c r="I18" s="21" t="s">
+      <c r="I18" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="J18" s="22" t="s">
+      <c r="J18" s="12" t="s">
         <v>263</v>
       </c>
-      <c r="K18" s="22" t="s">
+      <c r="K18" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="L18" s="22" t="s">
+      <c r="L18" s="12" t="s">
         <v>264</v>
       </c>
-      <c r="M18" s="22" t="s">
+      <c r="M18" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="N18" s="22" t="s">
+      <c r="N18" s="12" t="s">
         <v>265</v>
       </c>
-      <c r="O18" s="22" t="s">
+      <c r="O18" s="12" t="s">
         <v>266</v>
       </c>
-      <c r="P18" s="22" t="s">
+      <c r="P18" s="12" t="s">
         <v>267</v>
       </c>
-      <c r="Q18" s="22" t="s">
+      <c r="Q18" s="12" t="s">
         <v>268</v>
       </c>
-      <c r="R18" s="22" t="s">
+      <c r="R18" s="12" t="s">
         <v>269</v>
       </c>
-      <c r="S18" s="22" t="s">
+      <c r="S18" s="12" t="s">
         <v>270</v>
       </c>
-      <c r="T18" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="U18" s="21"/>
-      <c r="V18" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="W18" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="X18" s="21"/>
-      <c r="Y18" s="21"/>
-      <c r="Z18" s="23" t="n">
+      <c r="T18" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="U18" s="11"/>
+      <c r="V18" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="W18" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="X18" s="11"/>
+      <c r="Y18" s="11"/>
+      <c r="Z18" s="13" t="n">
         <v>42528350</v>
       </c>
-      <c r="AA18" s="24" t="s">
+      <c r="AA18" s="14" t="s">
         <v>271</v>
       </c>
-      <c r="AB18" s="22" t="s">
+      <c r="AB18" s="12" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="n">
+      <c r="A19" s="9" t="n">
         <v>15</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="C19" s="19" t="n">
+      <c r="C19" s="9" t="n">
         <v>2026</v>
       </c>
       <c r="D19" s="6" t="s">
@@ -5391,7 +5287,7 @@
       <c r="H19" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="I19" s="27" t="n">
+      <c r="I19" s="17" t="n">
         <v>0.57516339869281</v>
       </c>
       <c r="J19" s="6" t="s">
@@ -5424,20 +5320,20 @@
       <c r="S19" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="T19" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="U19" s="19"/>
-      <c r="V19" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="W19" s="19"/>
-      <c r="X19" s="19"/>
-      <c r="Y19" s="19"/>
-      <c r="Z19" s="25" t="n">
+      <c r="T19" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="U19" s="9"/>
+      <c r="V19" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W19" s="9"/>
+      <c r="X19" s="9"/>
+      <c r="Y19" s="9"/>
+      <c r="Z19" s="15" t="n">
         <v>42000525</v>
       </c>
-      <c r="AA19" s="20" t="s">
+      <c r="AA19" s="10" t="s">
         <v>287</v>
       </c>
       <c r="AB19" s="6" t="s">
@@ -5445,93 +5341,93 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="n">
+      <c r="A20" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="12" t="s">
         <v>289</v>
       </c>
-      <c r="C20" s="21" t="n">
+      <c r="C20" s="11" t="n">
         <v>2026</v>
       </c>
-      <c r="D20" s="22" t="s">
+      <c r="D20" s="12" t="s">
         <v>290</v>
       </c>
-      <c r="E20" s="22" t="s">
+      <c r="E20" s="12" t="s">
         <v>291</v>
       </c>
-      <c r="F20" s="22" t="s">
+      <c r="F20" s="12" t="s">
         <v>292</v>
       </c>
-      <c r="G20" s="22" t="s">
+      <c r="G20" s="12" t="s">
         <v>293</v>
       </c>
-      <c r="H20" s="22" t="s">
+      <c r="H20" s="12" t="s">
         <v>294</v>
       </c>
-      <c r="I20" s="21" t="s">
+      <c r="I20" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="J20" s="22" t="s">
+      <c r="J20" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="K20" s="22" t="s">
+      <c r="K20" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="L20" s="22" t="s">
+      <c r="L20" s="12" t="s">
         <v>295</v>
       </c>
-      <c r="M20" s="22" t="s">
+      <c r="M20" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="N20" s="22" t="s">
+      <c r="N20" s="12" t="s">
         <v>296</v>
       </c>
-      <c r="O20" s="22" t="s">
+      <c r="O20" s="12" t="s">
         <v>297</v>
       </c>
-      <c r="P20" s="22" t="s">
+      <c r="P20" s="12" t="s">
         <v>298</v>
       </c>
-      <c r="Q20" s="22" t="s">
+      <c r="Q20" s="12" t="s">
         <v>299</v>
       </c>
-      <c r="R20" s="22" t="s">
+      <c r="R20" s="12" t="s">
         <v>300</v>
       </c>
-      <c r="S20" s="22" t="s">
+      <c r="S20" s="12" t="s">
         <v>286</v>
       </c>
-      <c r="T20" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="U20" s="21"/>
-      <c r="V20" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="W20" s="21"/>
-      <c r="X20" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y20" s="21"/>
-      <c r="Z20" s="23" t="n">
+      <c r="T20" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="U20" s="11"/>
+      <c r="V20" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="W20" s="11"/>
+      <c r="X20" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y20" s="11"/>
+      <c r="Z20" s="13" t="n">
         <v>42614159</v>
       </c>
-      <c r="AA20" s="24" t="s">
+      <c r="AA20" s="14" t="s">
         <v>301</v>
       </c>
-      <c r="AB20" s="22" t="s">
+      <c r="AB20" s="12" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="n">
+      <c r="A21" s="9" t="n">
         <v>17</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>303</v>
       </c>
-      <c r="C21" s="19" t="n">
+      <c r="C21" s="9" t="n">
         <v>2023</v>
       </c>
       <c r="D21" s="6" t="s">
@@ -5549,7 +5445,7 @@
       <c r="H21" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="I21" s="27" t="n">
+      <c r="I21" s="17" t="n">
         <v>0.67</v>
       </c>
       <c r="J21" s="6" t="s">
@@ -5582,22 +5478,22 @@
       <c r="S21" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="T21" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="U21" s="19"/>
-      <c r="V21" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="W21" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="X21" s="19"/>
-      <c r="Y21" s="19"/>
-      <c r="Z21" s="25" t="n">
+      <c r="T21" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="U21" s="9"/>
+      <c r="V21" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W21" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="X21" s="9"/>
+      <c r="Y21" s="9"/>
+      <c r="Z21" s="15" t="n">
         <v>38075429</v>
       </c>
-      <c r="AA21" s="20" t="s">
+      <c r="AA21" s="10" t="s">
         <v>318</v>
       </c>
       <c r="AB21" s="6" t="s">
@@ -5605,91 +5501,91 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="n">
+      <c r="A22" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="12" t="s">
         <v>320</v>
       </c>
-      <c r="C22" s="21" t="n">
+      <c r="C22" s="11" t="n">
         <v>2022</v>
       </c>
-      <c r="D22" s="22" t="s">
+      <c r="D22" s="12" t="s">
         <v>321</v>
       </c>
-      <c r="E22" s="22" t="s">
+      <c r="E22" s="12" t="s">
         <v>322</v>
       </c>
-      <c r="F22" s="22" t="s">
+      <c r="F22" s="12" t="s">
         <v>323</v>
       </c>
-      <c r="G22" s="22" t="s">
+      <c r="G22" s="12" t="s">
         <v>324</v>
       </c>
-      <c r="H22" s="22" t="s">
+      <c r="H22" s="12" t="s">
         <v>325</v>
       </c>
-      <c r="I22" s="21" t="s">
+      <c r="I22" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="J22" s="22" t="s">
+      <c r="J22" s="12" t="s">
         <v>326</v>
       </c>
-      <c r="K22" s="22" t="s">
+      <c r="K22" s="12" t="s">
         <v>310</v>
       </c>
-      <c r="L22" s="22" t="s">
+      <c r="L22" s="12" t="s">
         <v>327</v>
       </c>
-      <c r="M22" s="22" t="s">
+      <c r="M22" s="12" t="s">
         <v>328</v>
       </c>
-      <c r="N22" s="22" t="s">
+      <c r="N22" s="12" t="s">
         <v>329</v>
       </c>
-      <c r="O22" s="22" t="s">
+      <c r="O22" s="12" t="s">
         <v>297</v>
       </c>
-      <c r="P22" s="22" t="s">
+      <c r="P22" s="12" t="s">
         <v>330</v>
       </c>
-      <c r="Q22" s="22" t="s">
+      <c r="Q22" s="12" t="s">
         <v>331</v>
       </c>
-      <c r="R22" s="22" t="s">
+      <c r="R22" s="12" t="s">
         <v>332</v>
       </c>
-      <c r="S22" s="22" t="s">
+      <c r="S22" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="T22" s="21"/>
-      <c r="U22" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="V22" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="W22" s="21"/>
-      <c r="X22" s="21"/>
-      <c r="Y22" s="21"/>
-      <c r="Z22" s="23" t="n">
+      <c r="T22" s="11"/>
+      <c r="U22" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="V22" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="W22" s="11"/>
+      <c r="X22" s="11"/>
+      <c r="Y22" s="11"/>
+      <c r="Z22" s="13" t="n">
         <v>36575415</v>
       </c>
-      <c r="AA22" s="24" t="s">
+      <c r="AA22" s="14" t="s">
         <v>334</v>
       </c>
-      <c r="AB22" s="22" t="s">
+      <c r="AB22" s="12" t="s">
         <v>335</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="n">
+      <c r="A23" s="9" t="n">
         <v>19</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>336</v>
       </c>
-      <c r="C23" s="19" t="n">
+      <c r="C23" s="9" t="n">
         <v>2026</v>
       </c>
       <c r="D23" s="6" t="s">
@@ -5707,7 +5603,7 @@
       <c r="H23" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="I23" s="27" t="n">
+      <c r="I23" s="17" t="n">
         <v>0.481481481481482</v>
       </c>
       <c r="J23" s="6" t="s">
@@ -5740,24 +5636,24 @@
       <c r="S23" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="T23" s="19"/>
-      <c r="U23" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="V23" s="19"/>
-      <c r="W23" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="X23" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y23" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z23" s="25" t="n">
+      <c r="T23" s="9"/>
+      <c r="U23" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V23" s="9"/>
+      <c r="W23" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="X23" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y23" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z23" s="15" t="n">
         <v>42305752</v>
       </c>
-      <c r="AA23" s="20" t="s">
+      <c r="AA23" s="10" t="s">
         <v>350</v>
       </c>
       <c r="AB23" s="6" t="s">
@@ -5765,87 +5661,87 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="n">
+      <c r="A24" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="12" t="s">
         <v>352</v>
       </c>
-      <c r="C24" s="21" t="n">
+      <c r="C24" s="11" t="n">
         <v>2023</v>
       </c>
-      <c r="D24" s="22" t="s">
+      <c r="D24" s="12" t="s">
         <v>353</v>
       </c>
-      <c r="E24" s="22" t="s">
+      <c r="E24" s="12" t="s">
         <v>354</v>
       </c>
-      <c r="F24" s="22" t="s">
+      <c r="F24" s="12" t="s">
         <v>355</v>
       </c>
-      <c r="G24" s="22" t="s">
+      <c r="G24" s="12" t="s">
         <v>356</v>
       </c>
-      <c r="H24" s="22" t="s">
+      <c r="H24" s="12" t="s">
         <v>357</v>
       </c>
-      <c r="I24" s="21" t="s">
+      <c r="I24" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="J24" s="22" t="s">
+      <c r="J24" s="12" t="s">
         <v>358</v>
       </c>
-      <c r="K24" s="22" t="s">
+      <c r="K24" s="12" t="s">
         <v>359</v>
       </c>
-      <c r="L24" s="22" t="s">
+      <c r="L24" s="12" t="s">
         <v>360</v>
       </c>
-      <c r="M24" s="22" t="s">
+      <c r="M24" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="N24" s="22" t="s">
+      <c r="N24" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="O24" s="22" t="s">
+      <c r="O24" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="P24" s="22" t="s">
+      <c r="P24" s="12" t="s">
         <v>361</v>
       </c>
-      <c r="Q24" s="22" t="s">
+      <c r="Q24" s="12" t="s">
         <v>362</v>
       </c>
-      <c r="R24" s="22" t="s">
+      <c r="R24" s="12" t="s">
         <v>363</v>
       </c>
-      <c r="S24" s="22" t="s">
+      <c r="S24" s="12" t="s">
         <v>349</v>
       </c>
-      <c r="T24" s="21"/>
-      <c r="U24" s="21"/>
-      <c r="V24" s="21"/>
-      <c r="W24" s="21"/>
-      <c r="X24" s="21"/>
-      <c r="Y24" s="21"/>
-      <c r="Z24" s="23" t="n">
+      <c r="T24" s="11"/>
+      <c r="U24" s="11"/>
+      <c r="V24" s="11"/>
+      <c r="W24" s="11"/>
+      <c r="X24" s="11"/>
+      <c r="Y24" s="11"/>
+      <c r="Z24" s="13" t="n">
         <v>36768099</v>
       </c>
-      <c r="AA24" s="24" t="s">
+      <c r="AA24" s="14" t="s">
         <v>364</v>
       </c>
-      <c r="AB24" s="22" t="s">
+      <c r="AB24" s="12" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="69" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="n">
+      <c r="A25" s="9" t="n">
         <v>21</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="C25" s="19" t="n">
+      <c r="C25" s="9" t="n">
         <v>2024</v>
       </c>
       <c r="D25" s="6" t="s">
@@ -5863,7 +5759,7 @@
       <c r="H25" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="I25" s="19" t="s">
+      <c r="I25" s="9" t="s">
         <v>14</v>
       </c>
       <c r="J25" s="6" t="s">
@@ -5896,20 +5792,20 @@
       <c r="S25" s="6" t="s">
         <v>376</v>
       </c>
-      <c r="T25" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="U25" s="19"/>
-      <c r="V25" s="19"/>
-      <c r="W25" s="19"/>
-      <c r="X25" s="19"/>
-      <c r="Y25" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z25" s="25" t="n">
+      <c r="T25" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="U25" s="9"/>
+      <c r="V25" s="9"/>
+      <c r="W25" s="9"/>
+      <c r="X25" s="9"/>
+      <c r="Y25" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z25" s="15" t="n">
         <v>38714782</v>
       </c>
-      <c r="AA25" s="20" t="s">
+      <c r="AA25" s="10" t="s">
         <v>377</v>
       </c>
       <c r="AB25" s="6" t="s">
@@ -5917,95 +5813,95 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="21" t="n">
+      <c r="A26" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="12" t="s">
         <v>379</v>
       </c>
-      <c r="C26" s="21" t="n">
+      <c r="C26" s="11" t="n">
         <v>2026</v>
       </c>
-      <c r="D26" s="22" t="s">
+      <c r="D26" s="12" t="s">
         <v>380</v>
       </c>
-      <c r="E26" s="22" t="s">
+      <c r="E26" s="12" t="s">
         <v>381</v>
       </c>
-      <c r="F26" s="22" t="s">
+      <c r="F26" s="12" t="s">
         <v>382</v>
       </c>
-      <c r="G26" s="22" t="s">
+      <c r="G26" s="12" t="s">
         <v>383</v>
       </c>
-      <c r="H26" s="22" t="s">
+      <c r="H26" s="12" t="s">
         <v>384</v>
       </c>
-      <c r="I26" s="26" t="n">
+      <c r="I26" s="16" t="n">
         <v>0.814</v>
       </c>
-      <c r="J26" s="22" t="s">
+      <c r="J26" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="K26" s="22" t="s">
+      <c r="K26" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="L26" s="22" t="s">
+      <c r="L26" s="12" t="s">
         <v>385</v>
       </c>
-      <c r="M26" s="22" t="s">
+      <c r="M26" s="12" t="s">
         <v>386</v>
       </c>
-      <c r="N26" s="22" t="s">
+      <c r="N26" s="12" t="s">
         <v>387</v>
       </c>
-      <c r="O26" s="22" t="s">
+      <c r="O26" s="12" t="s">
         <v>388</v>
       </c>
-      <c r="P26" s="22" t="s">
+      <c r="P26" s="12" t="s">
         <v>389</v>
       </c>
-      <c r="Q26" s="22" t="s">
+      <c r="Q26" s="12" t="s">
         <v>390</v>
       </c>
-      <c r="R26" s="22" t="s">
+      <c r="R26" s="12" t="s">
         <v>391</v>
       </c>
-      <c r="S26" s="22" t="s">
+      <c r="S26" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="T26" s="21"/>
-      <c r="U26" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="V26" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="W26" s="21"/>
-      <c r="X26" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y26" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z26" s="23" t="n">
+      <c r="T26" s="11"/>
+      <c r="U26" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="V26" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="W26" s="11"/>
+      <c r="X26" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y26" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z26" s="13" t="n">
         <v>42410881</v>
       </c>
-      <c r="AA26" s="24" t="s">
+      <c r="AA26" s="14" t="s">
         <v>392</v>
       </c>
-      <c r="AB26" s="22" t="s">
+      <c r="AB26" s="12" t="s">
         <v>393</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19" t="n">
+      <c r="A27" s="9" t="n">
         <v>23</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>394</v>
       </c>
-      <c r="C27" s="19" t="n">
+      <c r="C27" s="9" t="n">
         <v>2026</v>
       </c>
       <c r="D27" s="6" t="s">
@@ -6023,7 +5919,7 @@
       <c r="H27" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="I27" s="19" t="s">
+      <c r="I27" s="9" t="s">
         <v>16</v>
       </c>
       <c r="J27" s="6" t="s">
@@ -6056,20 +5952,20 @@
       <c r="S27" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="T27" s="19"/>
-      <c r="U27" s="19"/>
-      <c r="V27" s="19"/>
-      <c r="W27" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="X27" s="19"/>
-      <c r="Y27" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z27" s="25" t="n">
+      <c r="T27" s="9"/>
+      <c r="U27" s="9"/>
+      <c r="V27" s="9"/>
+      <c r="W27" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="X27" s="9"/>
+      <c r="Y27" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z27" s="15" t="n">
         <v>41911361</v>
       </c>
-      <c r="AA27" s="20" t="s">
+      <c r="AA27" s="10" t="s">
         <v>406</v>
       </c>
       <c r="AB27" s="6" t="s">
@@ -6077,95 +5973,95 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="21" t="n">
+      <c r="A28" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="12" t="s">
         <v>408</v>
       </c>
-      <c r="C28" s="21" t="n">
+      <c r="C28" s="11" t="n">
         <v>2026</v>
       </c>
-      <c r="D28" s="22" t="s">
+      <c r="D28" s="12" t="s">
         <v>409</v>
       </c>
-      <c r="E28" s="22" t="s">
+      <c r="E28" s="12" t="s">
         <v>410</v>
       </c>
-      <c r="F28" s="22" t="s">
+      <c r="F28" s="12" t="s">
         <v>411</v>
       </c>
-      <c r="G28" s="22" t="s">
+      <c r="G28" s="12" t="s">
         <v>412</v>
       </c>
-      <c r="H28" s="22" t="s">
+      <c r="H28" s="12" t="s">
         <v>413</v>
       </c>
-      <c r="I28" s="26" t="n">
+      <c r="I28" s="16" t="n">
         <v>0.315</v>
       </c>
-      <c r="J28" s="22" t="s">
+      <c r="J28" s="12" t="s">
         <v>414</v>
       </c>
-      <c r="K28" s="22" t="s">
+      <c r="K28" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="L28" s="22" t="s">
+      <c r="L28" s="12" t="s">
         <v>415</v>
       </c>
-      <c r="M28" s="22" t="s">
+      <c r="M28" s="12" t="s">
         <v>416</v>
       </c>
-      <c r="N28" s="22" t="s">
+      <c r="N28" s="12" t="s">
         <v>417</v>
       </c>
-      <c r="O28" s="22" t="s">
+      <c r="O28" s="12" t="s">
         <v>418</v>
       </c>
-      <c r="P28" s="22" t="s">
+      <c r="P28" s="12" t="s">
         <v>419</v>
       </c>
-      <c r="Q28" s="22" t="s">
+      <c r="Q28" s="12" t="s">
         <v>420</v>
       </c>
-      <c r="R28" s="22" t="s">
+      <c r="R28" s="12" t="s">
         <v>421</v>
       </c>
-      <c r="S28" s="22" t="s">
+      <c r="S28" s="12" t="s">
         <v>422</v>
       </c>
-      <c r="T28" s="21"/>
-      <c r="U28" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="V28" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="W28" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="X28" s="21"/>
-      <c r="Y28" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z28" s="23" t="n">
+      <c r="T28" s="11"/>
+      <c r="U28" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="V28" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="W28" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="X28" s="11"/>
+      <c r="Y28" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z28" s="13" t="n">
         <v>41876550</v>
       </c>
-      <c r="AA28" s="24" t="s">
+      <c r="AA28" s="14" t="s">
         <v>423</v>
       </c>
-      <c r="AB28" s="22" t="s">
+      <c r="AB28" s="12" t="s">
         <v>424</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="19" t="n">
+      <c r="A29" s="9" t="n">
         <v>25</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="C29" s="19" t="n">
+      <c r="C29" s="9" t="n">
         <v>2025</v>
       </c>
       <c r="D29" s="6" t="s">
@@ -6183,7 +6079,7 @@
       <c r="H29" s="6" t="s">
         <v>430</v>
       </c>
-      <c r="I29" s="19" t="s">
+      <c r="I29" s="9" t="s">
         <v>16</v>
       </c>
       <c r="J29" s="6" t="s">
@@ -6216,20 +6112,20 @@
       <c r="S29" s="6" t="s">
         <v>435</v>
       </c>
-      <c r="T29" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="U29" s="19"/>
-      <c r="V29" s="19"/>
-      <c r="W29" s="19"/>
-      <c r="X29" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y29" s="19"/>
-      <c r="Z29" s="25" t="n">
+      <c r="T29" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="U29" s="9"/>
+      <c r="V29" s="9"/>
+      <c r="W29" s="9"/>
+      <c r="X29" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y29" s="9"/>
+      <c r="Z29" s="15" t="n">
         <v>40145929</v>
       </c>
-      <c r="AA29" s="20" t="s">
+      <c r="AA29" s="10" t="s">
         <v>436</v>
       </c>
       <c r="AB29" s="6" t="s">
@@ -6237,95 +6133,95 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="21" t="n">
+      <c r="A30" s="11" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="22" t="s">
+      <c r="B30" s="12" t="s">
         <v>438</v>
       </c>
-      <c r="C30" s="21" t="n">
+      <c r="C30" s="11" t="n">
         <v>2024</v>
       </c>
-      <c r="D30" s="22" t="s">
+      <c r="D30" s="12" t="s">
         <v>439</v>
       </c>
-      <c r="E30" s="22" t="s">
+      <c r="E30" s="12" t="s">
         <v>440</v>
       </c>
-      <c r="F30" s="22" t="s">
+      <c r="F30" s="12" t="s">
         <v>441</v>
       </c>
-      <c r="G30" s="22" t="s">
+      <c r="G30" s="12" t="s">
         <v>442</v>
       </c>
-      <c r="H30" s="22" t="s">
+      <c r="H30" s="12" t="s">
         <v>443</v>
       </c>
-      <c r="I30" s="26" t="n">
+      <c r="I30" s="16" t="n">
         <v>0.719148936170213</v>
       </c>
-      <c r="J30" s="22" t="s">
+      <c r="J30" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="K30" s="22" t="s">
+      <c r="K30" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="L30" s="22" t="s">
+      <c r="L30" s="12" t="s">
         <v>444</v>
       </c>
-      <c r="M30" s="22" t="s">
+      <c r="M30" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="N30" s="22" t="s">
+      <c r="N30" s="12" t="s">
         <v>445</v>
       </c>
-      <c r="O30" s="22" t="s">
+      <c r="O30" s="12" t="s">
         <v>446</v>
       </c>
-      <c r="P30" s="22" t="s">
+      <c r="P30" s="12" t="s">
         <v>447</v>
       </c>
-      <c r="Q30" s="22" t="s">
+      <c r="Q30" s="12" t="s">
         <v>448</v>
       </c>
-      <c r="R30" s="22" t="s">
+      <c r="R30" s="12" t="s">
         <v>449</v>
       </c>
-      <c r="S30" s="22" t="s">
+      <c r="S30" s="12" t="s">
         <v>435</v>
       </c>
-      <c r="T30" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="U30" s="21"/>
-      <c r="V30" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="W30" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="X30" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y30" s="21"/>
-      <c r="Z30" s="23" t="n">
+      <c r="T30" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="U30" s="11"/>
+      <c r="V30" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="W30" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="X30" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y30" s="11"/>
+      <c r="Z30" s="13" t="n">
         <v>39439753</v>
       </c>
-      <c r="AA30" s="24" t="s">
+      <c r="AA30" s="14" t="s">
         <v>450</v>
       </c>
-      <c r="AB30" s="22" t="s">
+      <c r="AB30" s="12" t="s">
         <v>451</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="19" t="n">
+      <c r="A31" s="9" t="n">
         <v>27</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="C31" s="19" t="n">
+      <c r="C31" s="9" t="n">
         <v>2026</v>
       </c>
       <c r="D31" s="6" t="s">
@@ -6343,7 +6239,7 @@
       <c r="H31" s="6" t="s">
         <v>457</v>
       </c>
-      <c r="I31" s="27" t="n">
+      <c r="I31" s="17" t="n">
         <v>1</v>
       </c>
       <c r="J31" s="6" t="s">
@@ -6376,22 +6272,22 @@
       <c r="S31" s="6" t="s">
         <v>464</v>
       </c>
-      <c r="T31" s="19"/>
-      <c r="U31" s="19"/>
-      <c r="V31" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="W31" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="X31" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y31" s="19"/>
-      <c r="Z31" s="25" t="n">
+      <c r="T31" s="9"/>
+      <c r="U31" s="9"/>
+      <c r="V31" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W31" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="X31" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y31" s="9"/>
+      <c r="Z31" s="15" t="n">
         <v>41545627</v>
       </c>
-      <c r="AA31" s="20" t="s">
+      <c r="AA31" s="10" t="s">
         <v>465</v>
       </c>
       <c r="AB31" s="6" t="s">
@@ -6399,95 +6295,95 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="21" t="n">
+      <c r="A32" s="11" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="22" t="s">
+      <c r="B32" s="12" t="s">
         <v>467</v>
       </c>
-      <c r="C32" s="21" t="n">
+      <c r="C32" s="11" t="n">
         <v>2022</v>
       </c>
-      <c r="D32" s="22" t="s">
+      <c r="D32" s="12" t="s">
         <v>468</v>
       </c>
-      <c r="E32" s="22" t="s">
+      <c r="E32" s="12" t="s">
         <v>469</v>
       </c>
-      <c r="F32" s="22" t="s">
+      <c r="F32" s="12" t="s">
         <v>470</v>
       </c>
-      <c r="G32" s="22" t="s">
+      <c r="G32" s="12" t="s">
         <v>471</v>
       </c>
-      <c r="H32" s="22" t="s">
+      <c r="H32" s="12" t="s">
         <v>472</v>
       </c>
-      <c r="I32" s="26" t="n">
+      <c r="I32" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="J32" s="22" t="s">
+      <c r="J32" s="12" t="s">
         <v>473</v>
       </c>
-      <c r="K32" s="22" t="s">
+      <c r="K32" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="L32" s="22" t="s">
+      <c r="L32" s="12" t="s">
         <v>474</v>
       </c>
-      <c r="M32" s="22" t="s">
+      <c r="M32" s="12" t="s">
         <v>475</v>
       </c>
-      <c r="N32" s="22" t="s">
+      <c r="N32" s="12" t="s">
         <v>476</v>
       </c>
-      <c r="O32" s="22" t="s">
+      <c r="O32" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="P32" s="22" t="s">
+      <c r="P32" s="12" t="s">
         <v>477</v>
       </c>
-      <c r="Q32" s="22" t="s">
+      <c r="Q32" s="12" t="s">
         <v>478</v>
       </c>
-      <c r="R32" s="22" t="s">
+      <c r="R32" s="12" t="s">
         <v>479</v>
       </c>
-      <c r="S32" s="22" t="s">
+      <c r="S32" s="12" t="s">
         <v>435</v>
       </c>
-      <c r="T32" s="21"/>
-      <c r="U32" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="V32" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="W32" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="X32" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y32" s="21"/>
-      <c r="Z32" s="23" t="n">
+      <c r="T32" s="11"/>
+      <c r="U32" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="V32" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="W32" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="X32" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y32" s="11"/>
+      <c r="Z32" s="13" t="n">
         <v>35422659</v>
       </c>
-      <c r="AA32" s="24" t="s">
+      <c r="AA32" s="14" t="s">
         <v>480</v>
       </c>
-      <c r="AB32" s="22" t="s">
+      <c r="AB32" s="12" t="s">
         <v>481</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="19" t="n">
+      <c r="A33" s="9" t="n">
         <v>29</v>
       </c>
       <c r="B33" s="6" t="s">
         <v>482</v>
       </c>
-      <c r="C33" s="19" t="n">
+      <c r="C33" s="9" t="n">
         <v>2026</v>
       </c>
       <c r="D33" s="6" t="s">
@@ -6505,7 +6401,7 @@
       <c r="H33" s="6" t="s">
         <v>487</v>
       </c>
-      <c r="I33" s="19" t="s">
+      <c r="I33" s="9" t="s">
         <v>14</v>
       </c>
       <c r="J33" s="6" t="s">
@@ -6538,22 +6434,22 @@
       <c r="S33" s="6" t="s">
         <v>495</v>
       </c>
-      <c r="T33" s="19"/>
-      <c r="U33" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="V33" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="W33" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="X33" s="19"/>
-      <c r="Y33" s="19"/>
-      <c r="Z33" s="25" t="n">
+      <c r="T33" s="9"/>
+      <c r="U33" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V33" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W33" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="X33" s="9"/>
+      <c r="Y33" s="9"/>
+      <c r="Z33" s="15" t="n">
         <v>41065723</v>
       </c>
-      <c r="AA33" s="20" t="s">
+      <c r="AA33" s="10" t="s">
         <v>496</v>
       </c>
       <c r="AB33" s="6" t="s">
@@ -6561,93 +6457,93 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="21" t="n">
+      <c r="A34" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="22" t="s">
+      <c r="B34" s="12" t="s">
         <v>498</v>
       </c>
-      <c r="C34" s="21" t="n">
+      <c r="C34" s="11" t="n">
         <v>2026</v>
       </c>
-      <c r="D34" s="22" t="s">
+      <c r="D34" s="12" t="s">
         <v>499</v>
       </c>
-      <c r="E34" s="22" t="s">
+      <c r="E34" s="12" t="s">
         <v>500</v>
       </c>
-      <c r="F34" s="22" t="s">
+      <c r="F34" s="12" t="s">
         <v>501</v>
       </c>
-      <c r="G34" s="22" t="s">
+      <c r="G34" s="12" t="s">
         <v>502</v>
       </c>
-      <c r="H34" s="22" t="s">
+      <c r="H34" s="12" t="s">
         <v>503</v>
       </c>
-      <c r="I34" s="21" t="s">
+      <c r="I34" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="J34" s="22" t="s">
+      <c r="J34" s="12" t="s">
         <v>504</v>
       </c>
-      <c r="K34" s="22" t="s">
+      <c r="K34" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="L34" s="22" t="s">
+      <c r="L34" s="12" t="s">
         <v>505</v>
       </c>
-      <c r="M34" s="22" t="s">
+      <c r="M34" s="12" t="s">
         <v>506</v>
       </c>
-      <c r="N34" s="22" t="s">
+      <c r="N34" s="12" t="s">
         <v>507</v>
       </c>
-      <c r="O34" s="22" t="s">
+      <c r="O34" s="12" t="s">
         <v>508</v>
       </c>
-      <c r="P34" s="22" t="s">
+      <c r="P34" s="12" t="s">
         <v>509</v>
       </c>
-      <c r="Q34" s="22" t="s">
+      <c r="Q34" s="12" t="s">
         <v>510</v>
       </c>
-      <c r="R34" s="22" t="s">
+      <c r="R34" s="12" t="s">
         <v>511</v>
       </c>
-      <c r="S34" s="22" t="s">
+      <c r="S34" s="12" t="s">
         <v>495</v>
       </c>
-      <c r="T34" s="21"/>
-      <c r="U34" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="V34" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="W34" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="X34" s="21"/>
-      <c r="Y34" s="21"/>
-      <c r="Z34" s="23" t="n">
+      <c r="T34" s="11"/>
+      <c r="U34" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="V34" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="W34" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="X34" s="11"/>
+      <c r="Y34" s="11"/>
+      <c r="Z34" s="13" t="n">
         <v>42811329</v>
       </c>
-      <c r="AA34" s="24" t="s">
+      <c r="AA34" s="14" t="s">
         <v>512</v>
       </c>
-      <c r="AB34" s="22" t="s">
+      <c r="AB34" s="12" t="s">
         <v>513</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="19" t="n">
+      <c r="A35" s="9" t="n">
         <v>31</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>514</v>
       </c>
-      <c r="C35" s="19" t="n">
+      <c r="C35" s="9" t="n">
         <v>2025</v>
       </c>
       <c r="D35" s="6" t="s">
@@ -6665,7 +6561,7 @@
       <c r="H35" s="6" t="s">
         <v>518</v>
       </c>
-      <c r="I35" s="19" t="s">
+      <c r="I35" s="9" t="s">
         <v>14</v>
       </c>
       <c r="J35" s="6" t="s">
@@ -6698,22 +6594,22 @@
       <c r="S35" s="6" t="s">
         <v>526</v>
       </c>
-      <c r="T35" s="19"/>
-      <c r="U35" s="19"/>
-      <c r="V35" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="W35" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="X35" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y35" s="19"/>
-      <c r="Z35" s="25" t="n">
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W35" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="X35" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="15" t="n">
         <v>39788069</v>
       </c>
-      <c r="AA35" s="20" t="s">
+      <c r="AA35" s="10" t="s">
         <v>527</v>
       </c>
       <c r="AB35" s="6" t="s">
@@ -6721,95 +6617,95 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="21" t="n">
+      <c r="A36" s="11" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="22" t="s">
+      <c r="B36" s="12" t="s">
         <v>529</v>
       </c>
-      <c r="C36" s="21" t="n">
+      <c r="C36" s="11" t="n">
         <v>2025</v>
       </c>
-      <c r="D36" s="22" t="s">
+      <c r="D36" s="12" t="s">
         <v>530</v>
       </c>
-      <c r="E36" s="22" t="s">
+      <c r="E36" s="12" t="s">
         <v>531</v>
       </c>
-      <c r="F36" s="22" t="s">
+      <c r="F36" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="G36" s="22" t="s">
+      <c r="G36" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="H36" s="22" t="s">
+      <c r="H36" s="12" t="s">
         <v>532</v>
       </c>
-      <c r="I36" s="26" t="n">
+      <c r="I36" s="16" t="n">
         <v>0.84</v>
       </c>
-      <c r="J36" s="22" t="s">
+      <c r="J36" s="12" t="s">
         <v>533</v>
       </c>
-      <c r="K36" s="22" t="s">
+      <c r="K36" s="12" t="s">
         <v>310</v>
       </c>
-      <c r="L36" s="22" t="s">
+      <c r="L36" s="12" t="s">
         <v>534</v>
       </c>
-      <c r="M36" s="22" t="s">
+      <c r="M36" s="12" t="s">
         <v>535</v>
       </c>
-      <c r="N36" s="22" t="s">
+      <c r="N36" s="12" t="s">
         <v>536</v>
       </c>
-      <c r="O36" s="22" t="s">
+      <c r="O36" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="P36" s="22" t="s">
+      <c r="P36" s="12" t="s">
         <v>537</v>
       </c>
-      <c r="Q36" s="22" t="s">
+      <c r="Q36" s="12" t="s">
         <v>538</v>
       </c>
-      <c r="R36" s="22" t="s">
+      <c r="R36" s="12" t="s">
         <v>539</v>
       </c>
-      <c r="S36" s="22" t="s">
+      <c r="S36" s="12" t="s">
         <v>495</v>
       </c>
-      <c r="T36" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="U36" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="V36" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="W36" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="X36" s="21"/>
-      <c r="Y36" s="21"/>
-      <c r="Z36" s="23" t="n">
+      <c r="T36" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="U36" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="V36" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="W36" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="X36" s="11"/>
+      <c r="Y36" s="11"/>
+      <c r="Z36" s="13" t="n">
         <v>40370681</v>
       </c>
-      <c r="AA36" s="24" t="s">
+      <c r="AA36" s="14" t="s">
         <v>540</v>
       </c>
-      <c r="AB36" s="22" t="s">
+      <c r="AB36" s="12" t="s">
         <v>541</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="19" t="n">
+      <c r="A37" s="9" t="n">
         <v>33</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>542</v>
       </c>
-      <c r="C37" s="19" t="n">
+      <c r="C37" s="9" t="n">
         <v>2025</v>
       </c>
       <c r="D37" s="6" t="s">
@@ -6827,7 +6723,7 @@
       <c r="H37" s="6" t="s">
         <v>546</v>
       </c>
-      <c r="I37" s="19" t="s">
+      <c r="I37" s="9" t="s">
         <v>14</v>
       </c>
       <c r="J37" s="6" t="s">
@@ -6860,22 +6756,22 @@
       <c r="S37" s="6" t="s">
         <v>495</v>
       </c>
-      <c r="T37" s="19"/>
-      <c r="U37" s="19"/>
-      <c r="V37" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="W37" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="X37" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y37" s="19"/>
-      <c r="Z37" s="25" t="n">
+      <c r="T37" s="9"/>
+      <c r="U37" s="9"/>
+      <c r="V37" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W37" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="X37" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y37" s="9"/>
+      <c r="Z37" s="15" t="n">
         <v>41292097</v>
       </c>
-      <c r="AA37" s="20" t="s">
+      <c r="AA37" s="10" t="s">
         <v>555</v>
       </c>
       <c r="AB37" s="6" t="s">
@@ -6883,95 +6779,95 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="21" t="n">
+      <c r="A38" s="11" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="22" t="s">
+      <c r="B38" s="12" t="s">
         <v>557</v>
       </c>
-      <c r="C38" s="21" t="n">
+      <c r="C38" s="11" t="n">
         <v>2024</v>
       </c>
-      <c r="D38" s="22" t="s">
+      <c r="D38" s="12" t="s">
         <v>558</v>
       </c>
-      <c r="E38" s="22" t="s">
+      <c r="E38" s="12" t="s">
         <v>559</v>
       </c>
-      <c r="F38" s="22" t="s">
+      <c r="F38" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="G38" s="22" t="s">
+      <c r="G38" s="12" t="s">
         <v>560</v>
       </c>
-      <c r="H38" s="22" t="s">
+      <c r="H38" s="12" t="s">
         <v>561</v>
       </c>
-      <c r="I38" s="21" t="s">
+      <c r="I38" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="J38" s="22" t="s">
+      <c r="J38" s="12" t="s">
         <v>562</v>
       </c>
-      <c r="K38" s="22" t="s">
+      <c r="K38" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="L38" s="22" t="s">
+      <c r="L38" s="12" t="s">
         <v>563</v>
       </c>
-      <c r="M38" s="22" t="s">
+      <c r="M38" s="12" t="s">
         <v>564</v>
       </c>
-      <c r="N38" s="22" t="s">
+      <c r="N38" s="12" t="s">
         <v>565</v>
       </c>
-      <c r="O38" s="22" t="s">
+      <c r="O38" s="12" t="s">
         <v>566</v>
       </c>
-      <c r="P38" s="22" t="s">
+      <c r="P38" s="12" t="s">
         <v>567</v>
       </c>
-      <c r="Q38" s="22" t="s">
+      <c r="Q38" s="12" t="s">
         <v>568</v>
       </c>
-      <c r="R38" s="22" t="s">
+      <c r="R38" s="12" t="s">
         <v>569</v>
       </c>
-      <c r="S38" s="22" t="s">
+      <c r="S38" s="12" t="s">
         <v>495</v>
       </c>
-      <c r="T38" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="U38" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="V38" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="W38" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="X38" s="21"/>
-      <c r="Y38" s="21"/>
-      <c r="Z38" s="23" t="n">
+      <c r="T38" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="U38" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="V38" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="W38" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="X38" s="11"/>
+      <c r="Y38" s="11"/>
+      <c r="Z38" s="13" t="n">
         <v>38386373</v>
       </c>
-      <c r="AA38" s="24" t="s">
+      <c r="AA38" s="14" t="s">
         <v>570</v>
       </c>
-      <c r="AB38" s="22" t="s">
+      <c r="AB38" s="12" t="s">
         <v>571</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="19" t="n">
+      <c r="A39" s="9" t="n">
         <v>35</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>572</v>
       </c>
-      <c r="C39" s="19" t="n">
+      <c r="C39" s="9" t="n">
         <v>2024</v>
       </c>
       <c r="D39" s="6" t="s">
@@ -6989,7 +6885,7 @@
       <c r="H39" s="6" t="s">
         <v>576</v>
       </c>
-      <c r="I39" s="19" t="s">
+      <c r="I39" s="9" t="s">
         <v>14</v>
       </c>
       <c r="J39" s="6" t="s">
@@ -7022,24 +6918,24 @@
       <c r="S39" s="6" t="s">
         <v>495</v>
       </c>
-      <c r="T39" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="U39" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="V39" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="W39" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="X39" s="19"/>
-      <c r="Y39" s="19"/>
-      <c r="Z39" s="25" t="n">
+      <c r="T39" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="U39" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V39" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W39" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="X39" s="9"/>
+      <c r="Y39" s="9"/>
+      <c r="Z39" s="15" t="n">
         <v>38347557</v>
       </c>
-      <c r="AA39" s="20" t="s">
+      <c r="AA39" s="10" t="s">
         <v>585</v>
       </c>
       <c r="AB39" s="6" t="s">
@@ -7047,91 +6943,91 @@
       </c>
     </row>
     <row r="40" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="21" t="n">
+      <c r="A40" s="11" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="22" t="s">
+      <c r="B40" s="12" t="s">
         <v>587</v>
       </c>
-      <c r="C40" s="21" t="n">
+      <c r="C40" s="11" t="n">
         <v>2023</v>
       </c>
-      <c r="D40" s="22" t="s">
+      <c r="D40" s="12" t="s">
         <v>588</v>
       </c>
-      <c r="E40" s="22" t="s">
+      <c r="E40" s="12" t="s">
         <v>589</v>
       </c>
-      <c r="F40" s="22" t="s">
+      <c r="F40" s="12" t="s">
         <v>590</v>
       </c>
-      <c r="G40" s="22" t="s">
+      <c r="G40" s="12" t="s">
         <v>591</v>
       </c>
-      <c r="H40" s="22" t="s">
+      <c r="H40" s="12" t="s">
         <v>592</v>
       </c>
-      <c r="I40" s="26" t="n">
+      <c r="I40" s="16" t="n">
         <v>0.629</v>
       </c>
-      <c r="J40" s="22" t="s">
+      <c r="J40" s="12" t="s">
         <v>593</v>
       </c>
-      <c r="K40" s="22" t="s">
+      <c r="K40" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="L40" s="22" t="s">
+      <c r="L40" s="12" t="s">
         <v>594</v>
       </c>
-      <c r="M40" s="22" t="s">
+      <c r="M40" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="N40" s="22" t="s">
+      <c r="N40" s="12" t="s">
         <v>595</v>
       </c>
-      <c r="O40" s="22" t="s">
+      <c r="O40" s="12" t="s">
         <v>596</v>
       </c>
-      <c r="P40" s="22" t="s">
+      <c r="P40" s="12" t="s">
         <v>597</v>
       </c>
-      <c r="Q40" s="22" t="s">
+      <c r="Q40" s="12" t="s">
         <v>598</v>
       </c>
-      <c r="R40" s="22" t="s">
+      <c r="R40" s="12" t="s">
         <v>599</v>
       </c>
-      <c r="S40" s="22" t="s">
+      <c r="S40" s="12" t="s">
         <v>495</v>
       </c>
-      <c r="T40" s="21"/>
-      <c r="U40" s="21"/>
-      <c r="V40" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="W40" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="X40" s="21"/>
-      <c r="Y40" s="21"/>
-      <c r="Z40" s="23" t="n">
+      <c r="T40" s="11"/>
+      <c r="U40" s="11"/>
+      <c r="V40" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="W40" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="X40" s="11"/>
+      <c r="Y40" s="11"/>
+      <c r="Z40" s="13" t="n">
         <v>37143859</v>
       </c>
-      <c r="AA40" s="24" t="s">
+      <c r="AA40" s="14" t="s">
         <v>600</v>
       </c>
-      <c r="AB40" s="22" t="s">
+      <c r="AB40" s="12" t="s">
         <v>601</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="19" t="n">
+      <c r="A41" s="9" t="n">
         <v>37</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>602</v>
       </c>
-      <c r="C41" s="19" t="n">
+      <c r="C41" s="9" t="n">
         <v>2023</v>
       </c>
       <c r="D41" s="6" t="s">
@@ -7149,7 +7045,7 @@
       <c r="H41" s="6" t="s">
         <v>606</v>
       </c>
-      <c r="I41" s="27" t="n">
+      <c r="I41" s="17" t="n">
         <v>0.525</v>
       </c>
       <c r="J41" s="6" t="s">
@@ -7182,22 +7078,22 @@
       <c r="S41" s="6" t="s">
         <v>495</v>
       </c>
-      <c r="T41" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="U41" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="V41" s="19"/>
-      <c r="W41" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="X41" s="19"/>
-      <c r="Y41" s="19"/>
-      <c r="Z41" s="25" t="n">
+      <c r="T41" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="U41" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V41" s="9"/>
+      <c r="W41" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="X41" s="9"/>
+      <c r="Y41" s="9"/>
+      <c r="Z41" s="15" t="n">
         <v>37243855</v>
       </c>
-      <c r="AA41" s="20" t="s">
+      <c r="AA41" s="10" t="s">
         <v>614</v>
       </c>
       <c r="AB41" s="6" t="s">
@@ -7205,93 +7101,93 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="21" t="n">
+      <c r="A42" s="11" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="22" t="s">
+      <c r="B42" s="12" t="s">
         <v>616</v>
       </c>
-      <c r="C42" s="21" t="n">
+      <c r="C42" s="11" t="n">
         <v>2022</v>
       </c>
-      <c r="D42" s="22" t="s">
+      <c r="D42" s="12" t="s">
         <v>617</v>
       </c>
-      <c r="E42" s="22" t="s">
+      <c r="E42" s="12" t="s">
         <v>618</v>
       </c>
-      <c r="F42" s="22" t="s">
+      <c r="F42" s="12" t="s">
         <v>619</v>
       </c>
-      <c r="G42" s="22" t="s">
+      <c r="G42" s="12" t="s">
         <v>620</v>
       </c>
-      <c r="H42" s="22" t="s">
+      <c r="H42" s="12" t="s">
         <v>621</v>
       </c>
-      <c r="I42" s="26" t="n">
+      <c r="I42" s="16" t="n">
         <v>0.490566037735849</v>
       </c>
-      <c r="J42" s="22" t="s">
+      <c r="J42" s="12" t="s">
         <v>622</v>
       </c>
-      <c r="K42" s="22" t="s">
+      <c r="K42" s="12" t="s">
         <v>548</v>
       </c>
-      <c r="L42" s="22" t="s">
+      <c r="L42" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="M42" s="22" t="s">
+      <c r="M42" s="12" t="s">
         <v>623</v>
       </c>
-      <c r="N42" s="22" t="s">
+      <c r="N42" s="12" t="s">
         <v>624</v>
       </c>
-      <c r="O42" s="22" t="s">
+      <c r="O42" s="12" t="s">
         <v>625</v>
       </c>
-      <c r="P42" s="22" t="s">
+      <c r="P42" s="12" t="s">
         <v>626</v>
       </c>
-      <c r="Q42" s="22" t="s">
+      <c r="Q42" s="12" t="s">
         <v>627</v>
       </c>
-      <c r="R42" s="22" t="s">
+      <c r="R42" s="12" t="s">
         <v>628</v>
       </c>
-      <c r="S42" s="22" t="s">
+      <c r="S42" s="12" t="s">
         <v>495</v>
       </c>
-      <c r="T42" s="21"/>
-      <c r="U42" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="V42" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="W42" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="X42" s="21"/>
-      <c r="Y42" s="21"/>
-      <c r="Z42" s="23" t="n">
+      <c r="T42" s="11"/>
+      <c r="U42" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="V42" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="W42" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="X42" s="11"/>
+      <c r="Y42" s="11"/>
+      <c r="Z42" s="13" t="n">
         <v>36016077</v>
       </c>
-      <c r="AA42" s="24" t="s">
+      <c r="AA42" s="14" t="s">
         <v>629</v>
       </c>
-      <c r="AB42" s="22" t="s">
+      <c r="AB42" s="12" t="s">
         <v>630</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="19" t="n">
+      <c r="A43" s="9" t="n">
         <v>39</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>631</v>
       </c>
-      <c r="C43" s="19" t="n">
+      <c r="C43" s="9" t="n">
         <v>2021</v>
       </c>
       <c r="D43" s="6" t="s">
@@ -7309,7 +7205,7 @@
       <c r="H43" s="6" t="s">
         <v>634</v>
       </c>
-      <c r="I43" s="27" t="n">
+      <c r="I43" s="17" t="n">
         <v>0.647058823529412</v>
       </c>
       <c r="J43" s="6" t="s">
@@ -7342,20 +7238,20 @@
       <c r="S43" s="6" t="s">
         <v>495</v>
       </c>
-      <c r="T43" s="19"/>
-      <c r="U43" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="V43" s="19"/>
-      <c r="W43" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="X43" s="19"/>
-      <c r="Y43" s="19"/>
-      <c r="Z43" s="25" t="n">
+      <c r="T43" s="9"/>
+      <c r="U43" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V43" s="9"/>
+      <c r="W43" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="X43" s="9"/>
+      <c r="Y43" s="9"/>
+      <c r="Z43" s="15" t="n">
         <v>33378539</v>
       </c>
-      <c r="AA43" s="20" t="s">
+      <c r="AA43" s="10" t="s">
         <v>641</v>
       </c>
       <c r="AB43" s="6" t="s">
@@ -7363,91 +7259,91 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="21" t="n">
+      <c r="A44" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="22" t="s">
+      <c r="B44" s="12" t="s">
         <v>643</v>
       </c>
-      <c r="C44" s="21" t="n">
+      <c r="C44" s="11" t="n">
         <v>2025</v>
       </c>
-      <c r="D44" s="22" t="s">
+      <c r="D44" s="12" t="s">
         <v>644</v>
       </c>
-      <c r="E44" s="22" t="s">
+      <c r="E44" s="12" t="s">
         <v>381</v>
       </c>
-      <c r="F44" s="22" t="s">
+      <c r="F44" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="G44" s="22" t="s">
+      <c r="G44" s="12" t="s">
         <v>645</v>
       </c>
-      <c r="H44" s="22" t="s">
+      <c r="H44" s="12" t="s">
         <v>646</v>
       </c>
-      <c r="I44" s="26" t="n">
+      <c r="I44" s="16" t="n">
         <v>0.461538461538462</v>
       </c>
-      <c r="J44" s="22" t="s">
+      <c r="J44" s="12" t="s">
         <v>647</v>
       </c>
-      <c r="K44" s="22" t="s">
+      <c r="K44" s="12" t="s">
         <v>548</v>
       </c>
-      <c r="L44" s="22" t="s">
+      <c r="L44" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="M44" s="22" t="s">
+      <c r="M44" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="N44" s="22" t="s">
+      <c r="N44" s="12" t="s">
         <v>648</v>
       </c>
-      <c r="O44" s="22" t="s">
+      <c r="O44" s="12" t="s">
         <v>649</v>
       </c>
-      <c r="P44" s="22" t="s">
+      <c r="P44" s="12" t="s">
         <v>650</v>
       </c>
-      <c r="Q44" s="22" t="s">
+      <c r="Q44" s="12" t="s">
         <v>651</v>
       </c>
-      <c r="R44" s="22" t="s">
+      <c r="R44" s="12" t="s">
         <v>652</v>
       </c>
-      <c r="S44" s="22" t="s">
+      <c r="S44" s="12" t="s">
         <v>495</v>
       </c>
-      <c r="T44" s="21"/>
-      <c r="U44" s="21"/>
-      <c r="V44" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="W44" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="X44" s="21"/>
-      <c r="Y44" s="21"/>
-      <c r="Z44" s="23" t="n">
+      <c r="T44" s="11"/>
+      <c r="U44" s="11"/>
+      <c r="V44" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="W44" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="X44" s="11"/>
+      <c r="Y44" s="11"/>
+      <c r="Z44" s="13" t="n">
         <v>40834291</v>
       </c>
-      <c r="AA44" s="24" t="s">
+      <c r="AA44" s="14" t="s">
         <v>653</v>
       </c>
-      <c r="AB44" s="22" t="s">
+      <c r="AB44" s="12" t="s">
         <v>654</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="19" t="n">
+      <c r="A45" s="9" t="n">
         <v>41</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>587</v>
       </c>
-      <c r="C45" s="19" t="n">
+      <c r="C45" s="9" t="n">
         <v>2021</v>
       </c>
       <c r="D45" s="6" t="s">
@@ -7465,7 +7361,7 @@
       <c r="H45" s="6" t="s">
         <v>659</v>
       </c>
-      <c r="I45" s="27" t="n">
+      <c r="I45" s="17" t="n">
         <v>0.686868686868687</v>
       </c>
       <c r="J45" s="6" t="s">
@@ -7498,20 +7394,20 @@
       <c r="S45" s="6" t="s">
         <v>495</v>
       </c>
-      <c r="T45" s="19"/>
-      <c r="U45" s="19"/>
-      <c r="V45" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="W45" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="X45" s="19"/>
-      <c r="Y45" s="19"/>
-      <c r="Z45" s="25" t="n">
+      <c r="T45" s="9"/>
+      <c r="U45" s="9"/>
+      <c r="V45" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="W45" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="X45" s="9"/>
+      <c r="Y45" s="9"/>
+      <c r="Z45" s="15" t="n">
         <v>33529156</v>
       </c>
-      <c r="AA45" s="20" t="s">
+      <c r="AA45" s="10" t="s">
         <v>666</v>
       </c>
       <c r="AB45" s="6" t="s">
@@ -7529,7 +7425,7 @@
     <mergeCell ref="Z3:AB3"/>
   </mergeCells>
   <conditionalFormatting sqref="T5:Y45">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"Y"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7650,7 +7546,7 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="18" t="s">
         <v>670</v>
       </c>
       <c r="B4" s="7" t="s">
@@ -7661,66 +7557,66 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="19" t="s">
         <v>673</v>
       </c>
-      <c r="B5" s="30" t="n">
+      <c r="B5" s="20" t="n">
         <f aca="false">COUNTA('Literature Matrix'!$A$5:$A$45)</f>
         <v>41</v>
       </c>
-      <c r="C5" s="31"/>
+      <c r="C5" s="21"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="22" t="s">
         <v>674</v>
       </c>
-      <c r="B6" s="33" t="n">
+      <c r="B6" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$I$5:$I$45,"&gt;=0.5")</f>
         <v>12</v>
       </c>
-      <c r="C6" s="34" t="n">
+      <c r="C6" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B6/$B$5)</f>
         <v>0.292682926829268</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="22" t="s">
         <v>675</v>
       </c>
-      <c r="B7" s="33" t="n">
+      <c r="B7" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$I$5:$I$45,1)</f>
         <v>2</v>
       </c>
-      <c r="C7" s="34" t="n">
+      <c r="C7" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B7/$B$5)</f>
         <v>0.0487804878048781</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="22" t="s">
         <v>676</v>
       </c>
-      <c r="B8" s="33" t="n">
+      <c r="B8" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$I$5:$I$45,"NR")</f>
         <v>17</v>
       </c>
-      <c r="C8" s="34" t="n">
+      <c r="C8" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B8/$B$5)</f>
         <v>0.414634146341463</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="22" t="s">
         <v>677</v>
       </c>
-      <c r="B9" s="34" t="n">
+      <c r="B9" s="24" t="n">
         <f aca="false">IFERROR(AVERAGE('Literature Matrix'!$I$5:$I$45),0)</f>
         <v>0.657426614126057</v>
       </c>
-      <c r="C9" s="31"/>
+      <c r="C9" s="21"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28" t="s">
+      <c r="A11" s="18" t="s">
         <v>678</v>
       </c>
       <c r="B11" s="7" t="s">
@@ -7731,98 +7627,98 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="32" t="s">
+      <c r="A12" s="22" t="s">
         <v>679</v>
       </c>
-      <c r="B12" s="33" t="n">
+      <c r="B12" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$C$5:$C$45,2021)</f>
         <v>4</v>
       </c>
-      <c r="C12" s="34" t="n">
+      <c r="C12" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B12/$B$5)</f>
         <v>0.0975609756097561</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="22" t="s">
         <v>680</v>
       </c>
-      <c r="B13" s="33" t="n">
+      <c r="B13" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$C$5:$C$45,2022)</f>
         <v>4</v>
       </c>
-      <c r="C13" s="34" t="n">
+      <c r="C13" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B13/$B$5)</f>
         <v>0.0975609756097561</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="32" t="s">
+      <c r="A14" s="22" t="s">
         <v>681</v>
       </c>
-      <c r="B14" s="33" t="n">
+      <c r="B14" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$C$5:$C$45,2023)</f>
         <v>6</v>
       </c>
-      <c r="C14" s="34" t="n">
+      <c r="C14" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B14/$B$5)</f>
         <v>0.146341463414634</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="32" t="s">
+      <c r="A15" s="22" t="s">
         <v>682</v>
       </c>
-      <c r="B15" s="33" t="n">
+      <c r="B15" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$C$5:$C$45,2024)</f>
         <v>6</v>
       </c>
-      <c r="C15" s="34" t="n">
+      <c r="C15" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B15/$B$5)</f>
         <v>0.146341463414634</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="32" t="s">
+      <c r="A16" s="22" t="s">
         <v>683</v>
       </c>
-      <c r="B16" s="33" t="n">
+      <c r="B16" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$C$5:$C$45,2025)</f>
         <v>9</v>
       </c>
-      <c r="C16" s="34" t="n">
+      <c r="C16" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B16/$B$5)</f>
         <v>0.219512195121951</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="22" t="s">
         <v>684</v>
       </c>
-      <c r="B17" s="33" t="n">
+      <c r="B17" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$C$5:$C$45,2026)</f>
         <v>12</v>
       </c>
-      <c r="C17" s="34" t="n">
+      <c r="C17" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B17/$B$5)</f>
         <v>0.292682926829268</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29" t="s">
+      <c r="A18" s="19" t="s">
         <v>685</v>
       </c>
-      <c r="B18" s="30" t="n">
+      <c r="B18" s="20" t="n">
         <f aca="false">SUM(B12:B17)</f>
         <v>41</v>
       </c>
-      <c r="C18" s="34" t="n">
+      <c r="C18" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B18/$B$5)</f>
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="18" t="s">
         <v>686</v>
       </c>
       <c r="B20" s="7" t="s">
@@ -7833,124 +7729,124 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="32" t="s">
+      <c r="A21" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="B21" s="33" t="n">
+      <c r="B21" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$45,"Review")</f>
         <v>8</v>
       </c>
-      <c r="C21" s="34" t="n">
+      <c r="C21" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B21/$B$5)</f>
         <v>0.195121951219512</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="32" t="s">
+      <c r="A22" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="B22" s="33" t="n">
+      <c r="B22" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$45,"Cross-sectional")</f>
         <v>6</v>
       </c>
-      <c r="C22" s="34" t="n">
+      <c r="C22" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B22/$B$5)</f>
         <v>0.146341463414634</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="32" t="s">
+      <c r="A23" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="B23" s="33" t="n">
+      <c r="B23" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$45,"Longitudinal / cohort")</f>
         <v>12</v>
       </c>
-      <c r="C23" s="34" t="n">
+      <c r="C23" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B23/$B$5)</f>
         <v>0.292682926829268</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="32" t="s">
+      <c r="A24" s="22" t="s">
         <v>188</v>
       </c>
-      <c r="B24" s="33" t="n">
+      <c r="B24" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$45,"Daily diary / experience sampling")</f>
         <v>2</v>
       </c>
-      <c r="C24" s="34" t="n">
+      <c r="C24" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B24/$B$5)</f>
         <v>0.0487804878048781</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="32" t="s">
+      <c r="A25" s="22" t="s">
         <v>310</v>
       </c>
-      <c r="B25" s="33" t="n">
+      <c r="B25" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$45,"Intervention / quasi-experimental")</f>
         <v>4</v>
       </c>
-      <c r="C25" s="34" t="n">
+      <c r="C25" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B25/$B$5)</f>
         <v>0.0975609756097561</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="32" t="s">
+      <c r="A26" s="22" t="s">
         <v>548</v>
       </c>
-      <c r="B26" s="33" t="n">
+      <c r="B26" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$45,"Device validation")</f>
         <v>4</v>
       </c>
-      <c r="C26" s="34" t="n">
+      <c r="C26" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B26/$B$5)</f>
         <v>0.0975609756097561</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="32" t="s">
+      <c r="A27" s="22" t="s">
         <v>359</v>
       </c>
-      <c r="B27" s="33" t="n">
+      <c r="B27" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$45,"Measure validation")</f>
         <v>2</v>
       </c>
-      <c r="C27" s="34" t="n">
+      <c r="C27" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B27/$B$5)</f>
         <v>0.0487804878048781</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="32" t="s">
+      <c r="A28" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="B28" s="33" t="n">
+      <c r="B28" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$K$5:$K$45,"Other")</f>
         <v>3</v>
       </c>
-      <c r="C28" s="34" t="n">
+      <c r="C28" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B28/$B$5)</f>
         <v>0.0731707317073171</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="29" t="s">
+      <c r="A29" s="19" t="s">
         <v>685</v>
       </c>
-      <c r="B29" s="30" t="n">
+      <c r="B29" s="20" t="n">
         <f aca="false">SUM(B21:B28)</f>
         <v>41</v>
       </c>
-      <c r="C29" s="34" t="n">
+      <c r="C29" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B29/$B$5)</f>
         <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="28" t="s">
+      <c r="A31" s="18" t="s">
         <v>687</v>
       </c>
       <c r="B31" s="7" t="s">
@@ -7961,85 +7857,85 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="32" t="s">
+      <c r="A32" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="B32" s="33" t="n">
+      <c r="B32" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$T$5:$T$45,"Y")</f>
         <v>20</v>
       </c>
-      <c r="C32" s="34" t="n">
+      <c r="C32" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B32/$B$5)</f>
         <v>0.487804878048781</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="32" t="s">
+      <c r="A33" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="33" t="n">
+      <c r="B33" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$U$5:$U$45,"Y")</f>
         <v>21</v>
       </c>
-      <c r="C33" s="34" t="n">
+      <c r="C33" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B33/$B$5)</f>
         <v>0.51219512195122</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="32" t="s">
+      <c r="A34" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="B34" s="33" t="n">
+      <c r="B34" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$V$5:$V$45,"Y")</f>
         <v>23</v>
       </c>
-      <c r="C34" s="34" t="n">
+      <c r="C34" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B34/$B$5)</f>
         <v>0.560975609756098</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="32" t="s">
+      <c r="A35" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="B35" s="33" t="n">
+      <c r="B35" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$W$5:$W$45,"Y")</f>
         <v>23</v>
       </c>
-      <c r="C35" s="34" t="n">
+      <c r="C35" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B35/$B$5)</f>
         <v>0.560975609756098</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="32" t="s">
+      <c r="A36" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="B36" s="33" t="n">
+      <c r="B36" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$X$5:$X$45,"Y")</f>
         <v>12</v>
       </c>
-      <c r="C36" s="34" t="n">
+      <c r="C36" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B36/$B$5)</f>
         <v>0.292682926829268</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="32" t="s">
+      <c r="A37" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="B37" s="33" t="n">
+      <c r="B37" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$Y$5:$Y$45,"Y")</f>
         <v>9</v>
       </c>
-      <c r="C37" s="34" t="n">
+      <c r="C37" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B37/$B$5)</f>
         <v>0.219512195121951</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="28" t="s">
+      <c r="A39" s="18" t="s">
         <v>688</v>
       </c>
       <c r="B39" s="7" t="s">
@@ -8050,100 +7946,100 @@
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="32" t="s">
+      <c r="A40" s="22" t="s">
         <v>689</v>
       </c>
-      <c r="B40" s="33" t="n">
+      <c r="B40" s="23" t="n">
         <f aca="false">COUNTIFS('Literature Matrix'!$T$5:$T$45,"Y",'Literature Matrix'!$U$5:$U$45,"Y")</f>
         <v>10</v>
       </c>
-      <c r="C40" s="34" t="n">
+      <c r="C40" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B40/$B$5)</f>
         <v>0.24390243902439</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="32" t="s">
+      <c r="A41" s="22" t="s">
         <v>690</v>
       </c>
-      <c r="B41" s="33" t="n">
+      <c r="B41" s="23" t="n">
         <f aca="false">COUNTIFS('Literature Matrix'!$T$5:$T$45,"Y",'Literature Matrix'!$V$5:$V$45,"Y")</f>
         <v>9</v>
       </c>
-      <c r="C41" s="34" t="n">
+      <c r="C41" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B41/$B$5)</f>
         <v>0.219512195121951</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="32" t="s">
+      <c r="A42" s="22" t="s">
         <v>691</v>
       </c>
-      <c r="B42" s="33" t="n">
+      <c r="B42" s="23" t="n">
         <f aca="false">COUNTIFS('Literature Matrix'!$T$5:$T$45,"Y",'Literature Matrix'!$U$5:$U$45,"Y",'Literature Matrix'!$V$5:$V$45,"Y")</f>
         <v>4</v>
       </c>
-      <c r="C42" s="34" t="n">
+      <c r="C42" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B42/$B$5)</f>
         <v>0.0975609756097561</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="32" t="s">
+      <c r="A43" s="22" t="s">
         <v>692</v>
       </c>
-      <c r="B43" s="33" t="n">
+      <c r="B43" s="23" t="n">
         <f aca="false">COUNTIFS('Literature Matrix'!$T$5:$T$45,"Y",'Literature Matrix'!$U$5:$U$45,"Y",'Literature Matrix'!$V$5:$V$45,"Y",'Literature Matrix'!$W$5:$W$45,"Y")</f>
         <v>4</v>
       </c>
-      <c r="C43" s="34" t="n">
+      <c r="C43" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B43/$B$5)</f>
         <v>0.0975609756097561</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="32" t="s">
+      <c r="A44" s="22" t="s">
         <v>693</v>
       </c>
-      <c r="B44" s="33" t="n">
+      <c r="B44" s="23" t="n">
         <f aca="false">COUNTIFS('Literature Matrix'!$T$5:$T$45,"Y",'Literature Matrix'!$U$5:$U$45,"Y",'Literature Matrix'!$V$5:$V$45,"Y",'Literature Matrix'!$W$5:$W$45,"Y",'Literature Matrix'!$X$5:$X$45,"Y")</f>
         <v>0</v>
       </c>
-      <c r="C44" s="34" t="n">
+      <c r="C44" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B44/$B$5)</f>
         <v>0</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="32" t="s">
+      <c r="A45" s="22" t="s">
         <v>694</v>
       </c>
-      <c r="B45" s="33" t="n">
+      <c r="B45" s="23" t="n">
         <f aca="false">COUNTIFS('Literature Matrix'!$T$5:$T$45,"Y",'Literature Matrix'!$W$5:$W$45,"Y",'Literature Matrix'!$Y$5:$Y$45,"Y")</f>
         <v>0</v>
       </c>
-      <c r="C45" s="34" t="n">
+      <c r="C45" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B45/$B$5)</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="35" t="str">
+      <c r="A47" s="25" t="str">
         <f aca="false">"Gap: only "&amp;B43&amp;" of "&amp;B5&amp;" sources measured burnout, sleep, and HRV/RHR with a consumer wearable; "&amp;IF(B44=0,"none",B44)&amp;" of these reported results for women, and "&amp;IF(B45=0,"none",B45)&amp;" combined burnout and a consumer wearable in students."</f>
         <v>Gap: only 4 of 41 sources measured burnout, sleep, and HRV/RHR with a consumer wearable; none of these reported results for women, and none combined burnout and a consumer wearable in students.</v>
       </c>
-      <c r="B47" s="35"/>
-      <c r="C47" s="35"/>
+      <c r="B47" s="25"/>
+      <c r="C47" s="25"/>
     </row>
     <row r="48" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="36" t="s">
+      <c r="A48" s="26" t="s">
         <v>695</v>
       </c>
-      <c r="B48" s="36"/>
-      <c r="C48" s="36"/>
+      <c r="B48" s="26"/>
+      <c r="C48" s="26"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="28" t="s">
+      <c r="A50" s="18" t="s">
         <v>696</v>
       </c>
       <c r="B50" s="7" t="s">
@@ -8154,92 +8050,92 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="32" t="s">
+      <c r="A51" s="22" t="s">
         <v>697</v>
       </c>
-      <c r="B51" s="33" t="n">
+      <c r="B51" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$45,"*Oura*")</f>
         <v>6</v>
       </c>
-      <c r="C51" s="34" t="n">
+      <c r="C51" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B51/$B$5)</f>
         <v>0.146341463414634</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="32" t="s">
+      <c r="A52" s="22" t="s">
         <v>207</v>
       </c>
-      <c r="B52" s="33" t="n">
+      <c r="B52" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$45,"*Fitbit*")</f>
         <v>4</v>
       </c>
-      <c r="C52" s="34" t="n">
+      <c r="C52" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B52/$B$5)</f>
         <v>0.0975609756097561</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="32" t="s">
+      <c r="A53" s="22" t="s">
         <v>596</v>
       </c>
-      <c r="B53" s="33" t="n">
+      <c r="B53" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$45,"*Apple Watch*")</f>
         <v>3</v>
       </c>
-      <c r="C53" s="34" t="n">
+      <c r="C53" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B53/$B$5)</f>
         <v>0.0731707317073171</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="32" t="s">
+      <c r="A54" s="22" t="s">
         <v>698</v>
       </c>
-      <c r="B54" s="33" t="n">
+      <c r="B54" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$45,"*WHOOP*")</f>
         <v>4</v>
       </c>
-      <c r="C54" s="34" t="n">
+      <c r="C54" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B54/$B$5)</f>
         <v>0.0975609756097561</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="32" t="s">
+      <c r="A55" s="22" t="s">
         <v>699</v>
       </c>
-      <c r="B55" s="33" t="n">
+      <c r="B55" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$45,"*Garmin*")</f>
         <v>4</v>
       </c>
-      <c r="C55" s="34" t="n">
+      <c r="C55" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B55/$B$5)</f>
         <v>0.0975609756097561</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="32" t="s">
+      <c r="A56" s="22" t="s">
         <v>700</v>
       </c>
-      <c r="B56" s="33" t="n">
+      <c r="B56" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$45,"*Polar*")</f>
         <v>4</v>
       </c>
-      <c r="C56" s="34" t="n">
+      <c r="C56" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B56/$B$5)</f>
         <v>0.0975609756097561</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="32" t="s">
+      <c r="A57" s="22" t="s">
         <v>701</v>
       </c>
-      <c r="B57" s="33" t="n">
+      <c r="B57" s="23" t="n">
         <f aca="false">COUNTIF('Literature Matrix'!$O$5:$O$45,"*Huawei*")</f>
         <v>1</v>
       </c>
-      <c r="C57" s="34" t="n">
+      <c r="C57" s="24" t="n">
         <f aca="false">IF($B$5=0,0,B57/$B$5)</f>
         <v>0.024390243902439</v>
       </c>

</xml_diff>